<commit_message>
BOM and Head READMEs: whole 500 mm tube, no tube lock screw
The tube is used uncut and notched at its bottom end for the cables; the M4 x 6 tube-lock
set screw line is gone. The BOM and the Rev 4 and Rev 5 READMEs also carry the other
edits already in them.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/Heli_Collective_Final_BOM.xlsx
+++ b/BOM/Heli_Collective_Final_BOM.xlsx
@@ -633,7 +633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P78"/>
+  <dimension ref="A1:P79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2441,12 +2441,12 @@
       </c>
       <c r="O38" s="22" t="inlineStr">
         <is>
-          <t>In the set screw kit. From the boss's front (lower panel off): tap the 4.2 mm pilot M5; the tip pins the tube through the front wall of its 5.2 mm cross hole, 10 mm below the tube's top. Replaces the M5 x 40 bolt and nut (the kit's M5s stop at 20 mm)</t>
+          <t>In the set screw kit. From the boss's front (lower panel off), into its printed M5 thread; the tip pins the tube through the front wall of its 5.2 mm cross hole, 10 mm below the tube's top. Replaces the M5 x 40 bolt and nut (the kit's M5s stop at 20 mm)</t>
         </is>
       </c>
       <c r="P38" s="22" t="inlineStr">
         <is>
-          <t>HIQTRADEBYJJ set screw kit (Amazon B0DG33R714); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+          <t>HIQTRADEBYJJ set screw kit (Amazon B0DG33R714); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="P39" s="22" t="inlineStr">
         <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
         </is>
       </c>
     </row>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="P40" s="11" t="inlineStr">
         <is>
-          <t>Head/Rev4/README.md and Head/Rev3/README.md, Bought; Amazon listing 2026-10-23</t>
+          <t>Head/Rev5/README.md and Head/Rev4/README.md, Bought; Amazon listing 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -2638,12 +2638,12 @@
       </c>
       <c r="O41" s="11" t="inlineStr">
         <is>
-          <t>Ordered 2026-10-23. Uses the M3 x 25 (ISO 10642 / DIN 7991); the kits stop at 20 mm. Head in the countersink in the mount's left lug, through the trigger, then about 8 mm into the right lug's 2.5 mm pilot (tap it M3 all the way through); the tip stays about 0.9 mm inside the lug</t>
+          <t>Ordered 2026-10-23. Uses the M3 x 25 (ISO 10642 / DIN 7991); the kits stop at 20 mm. Head in the countersink in the mount's left lug, through the trigger, then about 8 mm into the right lug's printed M3 thread; the tip stays about 0.9 mm inside the lug</t>
         </is>
       </c>
       <c r="P41" s="11" t="inlineStr">
         <is>
-          <t>Head/Rev4/README.md and Head/Rev3/README.md, Bought; user's choice 2026-10-23; Amazon listing 2026-10-23</t>
+          <t>Head/Rev5/README.md and Head/Rev4/README.md, Bought; user's choice 2026-10-23; Amazon listing 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -2703,12 +2703,12 @@
       </c>
       <c r="O42" s="22" t="inlineStr">
         <is>
-          <t>In the set screw kit. Through the trigger's arm (tap M3); its tip bears on the mount. Set it so the starter switch clicks before the stop</t>
+          <t>In the set screw kit. Through the trigger's arm (printed M3 thread); its tip bears on the mount. Set it so the starter switch clicks before the stop</t>
         </is>
       </c>
       <c r="P42" s="22" t="inlineStr">
         <is>
-          <t>HIQTRADEBYJJ set screw kit (Amazon B0DG33R714); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+          <t>HIQTRADEBYJJ set screw kit (Amazon B0DG33R714); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
         </is>
       </c>
     </row>
@@ -2718,11 +2718,11 @@
       </c>
       <c r="B43" s="22" t="inlineStr">
         <is>
-          <t>Search hat bezel</t>
+          <t>Trigger pull stop seat</t>
         </is>
       </c>
       <c r="C43" s="21" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D43" s="21" t="n">
         <v>1</v>
@@ -2768,12 +2768,12 @@
       </c>
       <c r="O43" s="22" t="inlineStr">
         <is>
-          <t>In the screw kit. Through the hat's bezel into M2 threads tapped in the carrier (1.6 mm pilots)</t>
+          <t>In the screw kit. Flush in a countersunk, M2-tapped hole (1.6 mm pilot) in the mount's face under the spring pocket, so the pull stop's tip bears on steel and not on plastic</t>
         </is>
       </c>
       <c r="P43" s="22" t="inlineStr">
         <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
         </is>
       </c>
     </row>
@@ -2783,11 +2783,11 @@
       </c>
       <c r="B44" s="22" t="inlineStr">
         <is>
-          <t>Search hat pivot</t>
+          <t>Search hat bezel</t>
         </is>
       </c>
       <c r="C44" s="21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D44" s="21" t="n">
         <v>1</v>
@@ -2805,12 +2805,12 @@
       </c>
       <c r="H44" s="22" t="inlineStr">
         <is>
-          <t>M3 x 4 set screw</t>
+          <t>M2 x 8 countersunk screw</t>
         </is>
       </c>
       <c r="I44" s="22" t="inlineStr">
         <is>
-          <t>HIQTRADEBYJJ</t>
+          <t>AvrestYPT</t>
         </is>
       </c>
       <c r="J44" s="22" t="inlineStr"/>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="L44" s="24" t="inlineStr">
         <is>
-          <t>B0DG33R714</t>
+          <t>B0FMD5TMSH</t>
         </is>
       </c>
       <c r="M44" s="25" t="n">
@@ -2833,12 +2833,12 @@
       </c>
       <c r="O44" s="22" t="inlineStr">
         <is>
-          <t>In the set screw kit. Into the rocker plate's centre (tap M3), from behind; its tip is the pivot and sets the preload. Turn it with a 1.5 mm hex key through the carrier floor</t>
+          <t>In the screw kit. Through the hat's bezel into M2 threads tapped in the carrier (1.6 mm pilots)</t>
         </is>
       </c>
       <c r="P44" s="22" t="inlineStr">
         <is>
-          <t>HIQTRADEBYJJ set screw kit (Amazon B0DG33R714); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
         </is>
       </c>
     </row>
@@ -2848,11 +2848,11 @@
       </c>
       <c r="B45" s="22" t="inlineStr">
         <is>
-          <t>Panels</t>
+          <t>Search hat pivot</t>
         </is>
       </c>
       <c r="C45" s="21" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D45" s="21" t="n">
         <v>1</v>
@@ -2870,12 +2870,12 @@
       </c>
       <c r="H45" s="22" t="inlineStr">
         <is>
-          <t>M3 x 12 countersunk screw (DIN 7991)</t>
+          <t>M3 x 4 set screw</t>
         </is>
       </c>
       <c r="I45" s="22" t="inlineStr">
         <is>
-          <t>AvrestYPT</t>
+          <t>HIQTRADEBYJJ</t>
         </is>
       </c>
       <c r="J45" s="22" t="inlineStr"/>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="L45" s="24" t="inlineStr">
         <is>
-          <t>B0FMD5TMSH</t>
+          <t>B0DG33R714</t>
         </is>
       </c>
       <c r="M45" s="25" t="n">
@@ -2898,12 +2898,12 @@
       </c>
       <c r="O45" s="22" t="inlineStr">
         <is>
-          <t>In the screw kit. 4 per panel, into M3 threads tapped in the box's corner columns (the pilots run 50 mm deep, so the x 12 has room)</t>
+          <t>In the set screw kit. Into the rocker plate's centre (printed M3 thread), from behind; its tip is the pivot and sets the preload. Turn it with a 1.5 mm hex key through the carrier floor</t>
         </is>
       </c>
       <c r="P45" s="22" t="inlineStr">
         <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+          <t>HIQTRADEBYJJ set screw kit (Amazon B0DG33R714); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
         </is>
       </c>
     </row>
@@ -2913,11 +2913,11 @@
       </c>
       <c r="B46" s="22" t="inlineStr">
         <is>
-          <t>HeliSR board</t>
+          <t>Panels</t>
         </is>
       </c>
       <c r="C46" s="21" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D46" s="21" t="n">
         <v>1</v>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="H46" s="22" t="inlineStr">
         <is>
-          <t>M3 x 12 countersunk screw (DIN 7991) + M3 hex nut</t>
+          <t>M3 x 16 countersunk screw (DIN 7991)</t>
         </is>
       </c>
       <c r="I46" s="22" t="inlineStr">
@@ -2963,146 +2963,146 @@
       </c>
       <c r="O46" s="22" t="inlineStr">
         <is>
+          <t>In the screw kit. 4 per panel, into the M3 threads printed 20 mm deep in the box's corner columns (a kit M3 x 20 fits too)</t>
+        </is>
+      </c>
+      <c r="P46" s="22" t="inlineStr">
+        <is>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="21" t="n">
+        <v>31</v>
+      </c>
+      <c r="B47" s="22" t="inlineStr">
+        <is>
+          <t>HeliSR board</t>
+        </is>
+      </c>
+      <c r="C47" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="21">
+        <f>ROUNDUP(C47*$C$3/D47,0)</f>
+        <v/>
+      </c>
+      <c r="F47" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="21">
+        <f>MAX(0,E47-F47)</f>
+        <v/>
+      </c>
+      <c r="H47" s="22" t="inlineStr">
+        <is>
+          <t>M3 x 12 countersunk screw (DIN 7991) + M3 hex nut</t>
+        </is>
+      </c>
+      <c r="I47" s="22" t="inlineStr">
+        <is>
+          <t>AvrestYPT</t>
+        </is>
+      </c>
+      <c r="J47" s="22" t="inlineStr"/>
+      <c r="K47" s="22" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L47" s="24" t="inlineStr">
+        <is>
+          <t>B0FMD5TMSH</t>
+        </is>
+      </c>
+      <c r="M47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" s="25">
+        <f>IF(M47="","",G47*M47)</f>
+        <v/>
+      </c>
+      <c r="O47" s="22" t="inlineStr">
+        <is>
           <t>In the screw kit. From outside the rear wall through a spacer and the board</t>
         </is>
       </c>
-      <c r="P46" s="22" t="inlineStr">
-        <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="10" t="n">
-        <v>31</v>
-      </c>
-      <c r="B47" s="11" t="inlineStr">
+      <c r="P47" s="22" t="inlineStr">
+        <is>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
         <is>
           <t>HeliSR board</t>
         </is>
       </c>
-      <c r="C47" s="10" t="n">
+      <c r="C48" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="D47" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" s="10">
-        <f>ROUNDUP(C47*$C$3/D47,0)</f>
-        <v/>
-      </c>
-      <c r="F47" s="12" t="n">
+      <c r="D48" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="10">
+        <f>ROUNDUP(C48*$C$3/D48,0)</f>
+        <v/>
+      </c>
+      <c r="F48" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="G47" s="10">
-        <f>MAX(0,E47-F47)</f>
-        <v/>
-      </c>
-      <c r="H47" s="11" t="inlineStr">
+      <c r="G48" s="10">
+        <f>MAX(0,E48-F48)</f>
+        <v/>
+      </c>
+      <c r="H48" s="11" t="inlineStr">
         <is>
           <t>Round spacer, unthreaded, for M3, 4 mm long, 6.4 mm OD, PVC, self-retaining</t>
         </is>
       </c>
-      <c r="I47" s="11" t="inlineStr">
+      <c r="I48" s="11" t="inlineStr">
         <is>
           <t>Bivar</t>
         </is>
       </c>
-      <c r="J47" s="11" t="inlineStr">
+      <c r="J48" s="11" t="inlineStr">
         <is>
           <t>SRS-4-4MM</t>
         </is>
       </c>
-      <c r="K47" s="11" t="inlineStr">
+      <c r="K48" s="11" t="inlineStr">
         <is>
           <t>Digi-Key</t>
         </is>
       </c>
-      <c r="L47" s="13" t="inlineStr">
+      <c r="L48" s="13" t="inlineStr">
         <is>
           <t>SRS-4-4MM-ND</t>
         </is>
       </c>
-      <c r="M47" s="14" t="n">
+      <c r="M48" s="14" t="n">
         <v>0.1</v>
       </c>
-      <c r="N47" s="14">
-        <f>IF(M47="","",G47*M47)</f>
-        <v/>
-      </c>
-      <c r="O47" s="11" t="inlineStr">
+      <c r="N48" s="14">
+        <f>IF(M48="","",G48*M48)</f>
+        <v/>
+      </c>
+      <c r="O48" s="11" t="inlineStr">
         <is>
           <t>Between the rear wall and the board</t>
         </is>
       </c>
-      <c r="P47" s="11" t="inlineStr">
-        <is>
-          <t>Head/Rev4/README.md and Head/Rev3/README.md, Bought</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="26" t="n">
-        <v>32</v>
-      </c>
-      <c r="B48" s="27" t="inlineStr">
-        <is>
-          <t>Trigger</t>
-        </is>
-      </c>
-      <c r="C48" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="26" t="n">
-        <v>10</v>
-      </c>
-      <c r="E48" s="26">
-        <f>ROUNDUP(C48*$C$3/D48,0)</f>
-        <v/>
-      </c>
-      <c r="F48" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="26">
-        <f>MAX(0,E48-F48)</f>
-        <v/>
-      </c>
-      <c r="H48" s="27" t="inlineStr">
-        <is>
-          <t>Pen spring, 4 mm OD x 50 mm, 0.4 mm wire, pack of 10</t>
-        </is>
-      </c>
-      <c r="I48" s="27" t="inlineStr">
-        <is>
-          <t>uxcell</t>
-        </is>
-      </c>
-      <c r="J48" s="27" t="inlineStr"/>
-      <c r="K48" s="27" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="L48" s="29" t="inlineStr">
-        <is>
-          <t>B0GCZGNBYH</t>
-        </is>
-      </c>
-      <c r="M48" s="30" t="n">
-        <v>6.99</v>
-      </c>
-      <c r="N48" s="30">
-        <f>IF(M48="","",G48*M48)</f>
-        <v/>
-      </c>
-      <c r="O48" s="27" t="inlineStr">
-        <is>
-          <t>Trigger return: cut to about 13 mm</t>
-        </is>
-      </c>
-      <c r="P48" s="27" t="inlineStr">
-        <is>
-          <t>Head/Rev4/README.md and Head/Rev3/README.md, Bought; Amazon listing 2026-10-23</t>
+      <c r="P48" s="11" t="inlineStr">
+        <is>
+          <t>Head/Rev5/README.md and Head/Rev4/README.md, Bought</t>
         </is>
       </c>
     </row>
@@ -3112,14 +3112,14 @@
       </c>
       <c r="B49" s="27" t="inlineStr">
         <is>
-          <t>Head box</t>
+          <t>Trigger</t>
         </is>
       </c>
       <c r="C49" s="26" t="n">
         <v>1</v>
       </c>
       <c r="D49" s="26" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E49" s="26">
         <f>ROUNDUP(C49*$C$3/D49,0)</f>
@@ -3134,12 +3134,12 @@
       </c>
       <c r="H49" s="27" t="inlineStr">
         <is>
-          <t>Ballast: lead split shot fishing weights, assorted, 120 pcs</t>
+          <t>Pen spring, 4 mm OD x 50 mm, 0.4 mm wire, pack of 10</t>
         </is>
       </c>
       <c r="I49" s="27" t="inlineStr">
         <is>
-          <t>SANWEAL</t>
+          <t>uxcell</t>
         </is>
       </c>
       <c r="J49" s="27" t="inlineStr"/>
@@ -3150,11 +3150,11 @@
       </c>
       <c r="L49" s="29" t="inlineStr">
         <is>
-          <t>B0H6J3X6GL</t>
+          <t>B0GCZGNBYH</t>
         </is>
       </c>
       <c r="M49" s="30" t="n">
-        <v>5.99</v>
+        <v>6.99</v>
       </c>
       <c r="N49" s="30">
         <f>IF(M49="","",G49*M49)</f>
@@ -3162,116 +3162,112 @@
       </c>
       <c r="O49" s="27" t="inlineStr">
         <is>
+          <t>Trigger return: cut to about 13 mm</t>
+        </is>
+      </c>
+      <c r="P49" s="27" t="inlineStr">
+        <is>
+          <t>Head/Rev5/README.md and Head/Rev4/README.md, Bought; Amazon listing 2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="26" t="n">
+        <v>34</v>
+      </c>
+      <c r="B50" s="27" t="inlineStr">
+        <is>
+          <t>Head box</t>
+        </is>
+      </c>
+      <c r="C50" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="26">
+        <f>ROUNDUP(C50*$C$3/D50,0)</f>
+        <v/>
+      </c>
+      <c r="F50" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="26">
+        <f>MAX(0,E50-F50)</f>
+        <v/>
+      </c>
+      <c r="H50" s="27" t="inlineStr">
+        <is>
+          <t>Ballast: lead split shot fishing weights, assorted, 120 pcs</t>
+        </is>
+      </c>
+      <c r="I50" s="27" t="inlineStr">
+        <is>
+          <t>SANWEAL</t>
+        </is>
+      </c>
+      <c r="J50" s="27" t="inlineStr"/>
+      <c r="K50" s="27" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L50" s="29" t="inlineStr">
+        <is>
+          <t>B0H6J3X6GL</t>
+        </is>
+      </c>
+      <c r="M50" s="30" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="N50" s="30">
+        <f>IF(M50="","",G50*M50)</f>
+        <v/>
+      </c>
+      <c r="O50" s="27" t="inlineStr">
+        <is>
           <t>Only if the gas strut lifts too much: about 48 g for a 45 N strut. Close to the middle of the box. Weigh out what you need</t>
         </is>
       </c>
-      <c r="P49" s="27" t="inlineStr">
+      <c r="P50" s="27" t="inlineStr">
         <is>
           <t>Base/README.md, Bought parts; Amazon listing 2026-10-23</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="M50" s="3" t="inlineStr">
+    <row r="51">
+      <c r="M51" s="3" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="N50" s="15">
-        <f>SUM(N38:N49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="7" t="inlineStr">
+      <c r="N51" s="15">
+        <f>SUM(N38:N50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
         <is>
           <t>MkIII base Rev 3 (concept, not yet printed)</t>
         </is>
       </c>
-      <c r="B51" s="8" t="n"/>
-      <c r="C51" s="8" t="n"/>
-      <c r="D51" s="8" t="n"/>
-      <c r="E51" s="8" t="n"/>
-      <c r="F51" s="8" t="n"/>
-      <c r="G51" s="8" t="n"/>
-      <c r="H51" s="8" t="n"/>
-      <c r="I51" s="8" t="n"/>
-      <c r="J51" s="8" t="n"/>
-      <c r="K51" s="8" t="n"/>
-      <c r="L51" s="8" t="n"/>
-      <c r="M51" s="8" t="n"/>
-      <c r="N51" s="8" t="n"/>
-      <c r="O51" s="8" t="n"/>
-      <c r="P51" s="9" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="B52" s="11" t="inlineStr">
-        <is>
-          <t>Pivot</t>
-        </is>
-      </c>
-      <c r="C52" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D52" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E52" s="10">
-        <f>ROUNDUP(C52*$C$3/D52,0)</f>
-        <v/>
-      </c>
-      <c r="F52" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G52" s="10">
-        <f>MAX(0,E52-F52)</f>
-        <v/>
-      </c>
-      <c r="H52" s="11" t="inlineStr">
-        <is>
-          <t>Deep-groove ball bearing 6006-2RS, 30 x 55 x 13 mm</t>
-        </is>
-      </c>
-      <c r="I52" s="11" t="inlineStr">
-        <is>
-          <t>BlueStars</t>
-        </is>
-      </c>
-      <c r="J52" s="11" t="inlineStr">
-        <is>
-          <t>6006-2RS</t>
-        </is>
-      </c>
-      <c r="K52" s="11" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="L52" s="13" t="inlineStr">
-        <is>
-          <t>B09XTV8XYK</t>
-        </is>
-      </c>
-      <c r="M52" s="14" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="N52" s="14">
-        <f>IF(M52="","",G52*M52)</f>
-        <v/>
-      </c>
-      <c r="O52" s="11" t="inlineStr">
-        <is>
-          <t>Sold in pairs</t>
-        </is>
-      </c>
-      <c r="P52" s="11" t="inlineStr">
-        <is>
-          <t>Amazon listing on 2026-10-22 (link you sent); Base/mk3_pivot.py (the Rev 1 parts Rev 3 keeps)</t>
-        </is>
-      </c>
+      <c r="B52" s="8" t="n"/>
+      <c r="C52" s="8" t="n"/>
+      <c r="D52" s="8" t="n"/>
+      <c r="E52" s="8" t="n"/>
+      <c r="F52" s="8" t="n"/>
+      <c r="G52" s="8" t="n"/>
+      <c r="H52" s="8" t="n"/>
+      <c r="I52" s="8" t="n"/>
+      <c r="J52" s="8" t="n"/>
+      <c r="K52" s="8" t="n"/>
+      <c r="L52" s="8" t="n"/>
+      <c r="M52" s="8" t="n"/>
+      <c r="N52" s="8" t="n"/>
+      <c r="O52" s="8" t="n"/>
+      <c r="P52" s="9" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="n">
@@ -3279,11 +3275,11 @@
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>Tube</t>
+          <t>Pivot</t>
         </is>
       </c>
       <c r="C53" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D53" s="10" t="n">
         <v>2</v>
@@ -3301,15 +3297,19 @@
       </c>
       <c r="H53" s="11" t="inlineStr">
         <is>
-          <t>Carbon fibre tube, 25 mm OD x 23 mm ID, 500 mm, 3K plain weave, wrapped</t>
+          <t>Deep-groove ball bearing 6006-2RS, 30 x 55 x 13 mm</t>
         </is>
       </c>
       <c r="I53" s="11" t="inlineStr">
         <is>
-          <t>MECCANIXITY</t>
-        </is>
-      </c>
-      <c r="J53" s="11" t="inlineStr"/>
+          <t>BlueStars</t>
+        </is>
+      </c>
+      <c r="J53" s="11" t="inlineStr">
+        <is>
+          <t>6006-2RS</t>
+        </is>
+      </c>
       <c r="K53" s="11" t="inlineStr">
         <is>
           <t>Amazon</t>
@@ -3317,11 +3317,11 @@
       </c>
       <c r="L53" s="13" t="inlineStr">
         <is>
-          <t>B0CFFT1B31</t>
+          <t>B09XTV8XYK</t>
         </is>
       </c>
       <c r="M53" s="14" t="n">
-        <v>27.49</v>
+        <v>8.99</v>
       </c>
       <c r="N53" s="14">
         <f>IF(M53="","",G53*M53)</f>
@@ -3329,207 +3329,207 @@
       </c>
       <c r="O53" s="11" t="inlineStr">
         <is>
-          <t>Sold in pairs. Wrapped, as the base needs (not pultruded). Cut to 491 mm (470 + the head's extra 12.7 mm of bore + 8 mm for the base's deeper socket). Drill the M4 lock-screw hole 38.5 mm from the bottom end and the head's 5.2 mm cross hole 10 mm below the top end. Check the socket and head fits with it (coupons)</t>
+          <t>Sold in pairs</t>
         </is>
       </c>
       <c r="P53" s="11" t="inlineStr">
         <is>
+          <t>Amazon listing on 2026-10-22 (link you sent); Base/mk3_pivot.py (the Rev 1 parts Rev 3 keeps)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>Tube</t>
+        </is>
+      </c>
+      <c r="C54" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" s="10">
+        <f>ROUNDUP(C54*$C$3/D54,0)</f>
+        <v/>
+      </c>
+      <c r="F54" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="10">
+        <f>MAX(0,E54-F54)</f>
+        <v/>
+      </c>
+      <c r="H54" s="11" t="inlineStr">
+        <is>
+          <t>Carbon fibre tube, 25 mm OD x 23 mm ID, 500 mm, 3K plain weave, wrapped</t>
+        </is>
+      </c>
+      <c r="I54" s="11" t="inlineStr">
+        <is>
+          <t>MECCANIXITY</t>
+        </is>
+      </c>
+      <c r="J54" s="11" t="inlineStr"/>
+      <c r="K54" s="11" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L54" s="13" t="inlineStr">
+        <is>
+          <t>B0CFFT1B31</t>
+        </is>
+      </c>
+      <c r="M54" s="14" t="n">
+        <v>27.49</v>
+      </c>
+      <c r="N54" s="14">
+        <f>IF(M54="","",G54*M54)</f>
+        <v/>
+      </c>
+      <c r="O54" s="11" t="inlineStr">
+        <is>
+          <t>Sold in pairs. Wrapped, as the base needs (not pultruded). Used whole, 500 mm, uncut (470 + the head's extra 12.7 mm of bore + 17.3 mm down in the base's socket). Drill the head's 5.2 mm cross hole 10 mm below the top end and file a 13 mm wide notch, 4+ mm deep, in each side of the bottom end for the cables. Check the socket and head fits with it (coupons)</t>
+        </is>
+      </c>
+      <c r="P54" s="11" t="inlineStr">
+        <is>
           <t>Amazon listing on 2026-10-22 (link you sent); Base/README.md, Bought parts</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="21" t="n">
-        <v>36</v>
-      </c>
-      <c r="B54" s="22" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="21" t="n">
+        <v>37</v>
+      </c>
+      <c r="B55" s="22" t="inlineStr">
         <is>
           <t>Lever halves</t>
         </is>
       </c>
-      <c r="C54" s="21" t="n">
+      <c r="C55" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="D54" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" s="21">
-        <f>ROUNDUP(C54*$C$3/D54,0)</f>
-        <v/>
-      </c>
-      <c r="F54" s="23" t="n">
+      <c r="D55" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="21">
+        <f>ROUNDUP(C55*$C$3/D55,0)</f>
+        <v/>
+      </c>
+      <c r="F55" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G54" s="21">
-        <f>MAX(0,E54-F54)</f>
-        <v/>
-      </c>
-      <c r="H54" s="22" t="inlineStr">
+      <c r="G55" s="21">
+        <f>MAX(0,E55-F55)</f>
+        <v/>
+      </c>
+      <c r="H55" s="22" t="inlineStr">
         <is>
           <t>M4 x 20 countersunk screw + M4 hex nut</t>
         </is>
       </c>
-      <c r="I54" s="22" t="inlineStr">
+      <c r="I55" s="22" t="inlineStr">
         <is>
           <t>AvrestYPT</t>
         </is>
       </c>
-      <c r="J54" s="22" t="inlineStr"/>
-      <c r="K54" s="22" t="inlineStr">
+      <c r="J55" s="22" t="inlineStr"/>
+      <c r="K55" s="22" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="L54" s="24" t="inlineStr">
+      <c r="L55" s="24" t="inlineStr">
         <is>
           <t>B0FMD5TMSH</t>
         </is>
       </c>
-      <c r="M54" s="25" t="n">
+      <c r="M55" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="N54" s="25">
-        <f>IF(M54="","",G54*M54)</f>
-        <v/>
-      </c>
-      <c r="O54" s="22" t="inlineStr">
+      <c r="N55" s="25">
+        <f>IF(M55="","",G55*M55)</f>
+        <v/>
+      </c>
+      <c r="O55" s="22" t="inlineStr">
         <is>
           <t>In the screw kit. From the top, the heads 16 mm down their counterbores (a long 2.5 mm hex key helps); the nuts go in the lower half's pockets first</t>
         </is>
       </c>
-      <c r="P54" s="22" t="inlineStr">
-        <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="10" t="n">
-        <v>37</v>
-      </c>
-      <c r="B55" s="11" t="inlineStr">
+      <c r="P55" s="22" t="inlineStr">
+        <is>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
         <is>
           <t>Strut</t>
         </is>
       </c>
-      <c r="C55" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" s="10" t="n">
+      <c r="C56" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E55" s="10">
-        <f>ROUNDUP(C55*$C$3/D55,0)</f>
-        <v/>
-      </c>
-      <c r="F55" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G55" s="10">
-        <f>MAX(0,E55-F55)</f>
-        <v/>
-      </c>
-      <c r="H55" s="11" t="inlineStr">
+      <c r="E56" s="10">
+        <f>ROUNDUP(C56*$C$3/D56,0)</f>
+        <v/>
+      </c>
+      <c r="F56" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="10">
+        <f>MAX(0,E56-F56)</f>
+        <v/>
+      </c>
+      <c r="H56" s="11" t="inlineStr">
         <is>
           <t>Gas strut, 6 in (152.4 mm eye to eye), 45 N (sold as 9-12 lb), flat eyelet tabs</t>
         </is>
       </c>
-      <c r="I55" s="11" t="inlineStr">
+      <c r="I56" s="11" t="inlineStr">
         <is>
           <t>X AUTOHAUX</t>
         </is>
       </c>
-      <c r="J55" s="11" t="inlineStr"/>
-      <c r="K55" s="11" t="inlineStr">
+      <c r="J56" s="11" t="inlineStr"/>
+      <c r="K56" s="11" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="L55" s="13" t="inlineStr">
+      <c r="L56" s="13" t="inlineStr">
         <is>
           <t>B0CY267GFY</t>
         </is>
       </c>
-      <c r="M55" s="14" t="n">
+      <c r="M56" s="14" t="n">
         <v>13.69</v>
       </c>
-      <c r="N55" s="14">
-        <f>IF(M55="","",G55*M55)</f>
-        <v/>
-      </c>
-      <c r="O55" s="11" t="inlineStr">
+      <c r="N56" s="14">
+        <f>IF(M56="","",G56*M56)</f>
+        <v/>
+      </c>
+      <c r="O56" s="11" t="inlineStr">
         <is>
           <t>Sold in pairs: the spare is the other half</t>
         </is>
       </c>
-      <c r="P55" s="11" t="inlineStr">
+      <c r="P56" s="11" t="inlineStr">
         <is>
           <t>Base/README.md, Bought parts</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="21" t="n">
-        <v>38</v>
-      </c>
-      <c r="B56" s="22" t="inlineStr">
-        <is>
-          <t>Strut eyes</t>
-        </is>
-      </c>
-      <c r="C56" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="D56" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="21">
-        <f>ROUNDUP(C56*$C$3/D56,0)</f>
-        <v/>
-      </c>
-      <c r="F56" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="21">
-        <f>MAX(0,E56-F56)</f>
-        <v/>
-      </c>
-      <c r="H56" s="22" t="inlineStr">
-        <is>
-          <t>M4 x 16 countersunk screw + M4 hex nut</t>
-        </is>
-      </c>
-      <c r="I56" s="22" t="inlineStr">
-        <is>
-          <t>AvrestYPT</t>
-        </is>
-      </c>
-      <c r="J56" s="22" t="inlineStr"/>
-      <c r="K56" s="22" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="L56" s="24" t="inlineStr">
-        <is>
-          <t>B0FMD5TMSH</t>
-        </is>
-      </c>
-      <c r="M56" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N56" s="25">
-        <f>IF(M56="","",G56*M56)</f>
-        <v/>
-      </c>
-      <c r="O56" s="22" t="inlineStr">
-        <is>
-          <t>In the screw kit. One per eye: head on +y, nut in the -y cheek's pocket. The listing gives the strut's eye holes as 4 mm. Snug, then thread-lock: the eye must still turn</t>
-        </is>
-      </c>
-      <c r="P56" s="22" t="inlineStr">
-        <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
         </is>
       </c>
     </row>
@@ -3539,11 +3539,11 @@
       </c>
       <c r="B57" s="22" t="inlineStr">
         <is>
-          <t>Strut collar</t>
+          <t>Strut eyes</t>
         </is>
       </c>
       <c r="C57" s="21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D57" s="21" t="n">
         <v>1</v>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="H57" s="22" t="inlineStr">
         <is>
-          <t>M4 x 12 countersunk screw + M4 hex nut</t>
+          <t>M4 x 16 countersunk screw + M4 hex nut</t>
         </is>
       </c>
       <c r="I57" s="22" t="inlineStr">
@@ -3589,12 +3589,12 @@
       </c>
       <c r="O57" s="22" t="inlineStr">
         <is>
-          <t>In the screw kit. Collar clamp: the head sits 2 mm into the -y ear, the nut in the +y ear's pocket</t>
+          <t>In the screw kit. One per eye: head on +y, nut in the -y cheek's pocket. The listing gives the strut's eye holes as 4 mm. Snug, then thread-lock: the eye must still turn</t>
         </is>
       </c>
       <c r="P57" s="22" t="inlineStr">
         <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
         </is>
       </c>
     </row>
@@ -3604,11 +3604,11 @@
       </c>
       <c r="B58" s="22" t="inlineStr">
         <is>
-          <t>Down-stops</t>
+          <t>Strut collar</t>
         </is>
       </c>
       <c r="C58" s="21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D58" s="21" t="n">
         <v>1</v>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="H58" s="22" t="inlineStr">
         <is>
-          <t>M4 x 16 countersunk screw + 2 M4 hex nuts</t>
+          <t>M4 x 12 countersunk screw + M4 hex nut</t>
         </is>
       </c>
       <c r="I58" s="22" t="inlineStr">
@@ -3654,12 +3654,12 @@
       </c>
       <c r="O58" s="22" t="inlineStr">
         <is>
-          <t>In the screw kit. Head up: its flat top is the stop. One nut pressed into the post's top pocket, the second on top of it locks the height that levels the tube</t>
+          <t>In the screw kit. Collar clamp: the head sits 2 mm into the -y ear, the nut in the +y ear's pocket</t>
         </is>
       </c>
       <c r="P58" s="22" t="inlineStr">
         <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
         </is>
       </c>
     </row>
@@ -3669,11 +3669,11 @@
       </c>
       <c r="B59" s="22" t="inlineStr">
         <is>
-          <t>Pillow-block caps</t>
+          <t>Down-stops</t>
         </is>
       </c>
       <c r="C59" s="21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D59" s="21" t="n">
         <v>1</v>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="H59" s="22" t="inlineStr">
         <is>
-          <t>M4 x 20 countersunk screw + M4 hex nut</t>
+          <t>M4 x 16 countersunk screw + 2 M4 hex nuts</t>
         </is>
       </c>
       <c r="I59" s="22" t="inlineStr">
@@ -3719,144 +3719,144 @@
       </c>
       <c r="O59" s="22" t="inlineStr">
         <is>
+          <t>In the screw kit. Head up: its flat top is the stop. One nut pressed into the post's top pocket, the second on top of it locks the height that levels the tube</t>
+        </is>
+      </c>
+      <c r="P59" s="22" t="inlineStr">
+        <is>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="21" t="n">
+        <v>42</v>
+      </c>
+      <c r="B60" s="22" t="inlineStr">
+        <is>
+          <t>Pillow-block caps</t>
+        </is>
+      </c>
+      <c r="C60" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D60" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="21">
+        <f>ROUNDUP(C60*$C$3/D60,0)</f>
+        <v/>
+      </c>
+      <c r="F60" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="21">
+        <f>MAX(0,E60-F60)</f>
+        <v/>
+      </c>
+      <c r="H60" s="22" t="inlineStr">
+        <is>
+          <t>M4 x 20 countersunk screw + M4 hex nut</t>
+        </is>
+      </c>
+      <c r="I60" s="22" t="inlineStr">
+        <is>
+          <t>AvrestYPT</t>
+        </is>
+      </c>
+      <c r="J60" s="22" t="inlineStr"/>
+      <c r="K60" s="22" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L60" s="24" t="inlineStr">
+        <is>
+          <t>B0FMD5TMSH</t>
+        </is>
+      </c>
+      <c r="M60" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" s="25">
+        <f>IF(M60="","",G60*M60)</f>
+        <v/>
+      </c>
+      <c r="O60" s="22" t="inlineStr">
+        <is>
           <t>In the screw kit. Two per cap, from the top; each nut slides into a slot in the block's front or back face. Length from the CAD</t>
         </is>
       </c>
-      <c r="P59" s="22" t="inlineStr">
-        <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="B60" s="11" t="inlineStr">
+      <c r="P60" s="22" t="inlineStr">
+        <is>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
         <is>
           <t>Side covers</t>
         </is>
       </c>
-      <c r="C60" s="10" t="n">
+      <c r="C61" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="D60" s="10" t="inlineStr">
+      <c r="D61" s="10" t="inlineStr">
         <is>
           <t>once</t>
         </is>
       </c>
-      <c r="E60" s="10">
-        <f>IF($C$3&gt;0,C60,0)</f>
-        <v/>
-      </c>
-      <c r="F60" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G60" s="10">
-        <f>MAX(0,E60-F60)</f>
-        <v/>
-      </c>
-      <c r="H60" s="11" t="inlineStr">
+      <c r="E61" s="10">
+        <f>IF($C$3&gt;0,C61,0)</f>
+        <v/>
+      </c>
+      <c r="F61" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="10">
+        <f>MAX(0,E61-F61)</f>
+        <v/>
+      </c>
+      <c r="H61" s="11" t="inlineStr">
         <is>
           <t>M3 x 25 countersunk screw (from the M3 x 20-40 set, ASIN B0BYXS4BTF)</t>
         </is>
       </c>
-      <c r="I60" s="11" t="inlineStr">
+      <c r="I61" s="11" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="J60" s="11" t="inlineStr"/>
-      <c r="K60" s="11" t="inlineStr">
+      <c r="J61" s="11" t="inlineStr"/>
+      <c r="K61" s="11" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="L60" s="13" t="inlineStr">
+      <c r="L61" s="13" t="inlineStr">
         <is>
           <t>B0BYXS4BTF</t>
         </is>
       </c>
-      <c r="M60" s="14" t="n">
+      <c r="M61" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N60" s="14">
-        <f>IF(M60="","",G60*M60)</f>
-        <v/>
-      </c>
-      <c r="O60" s="11" t="inlineStr">
+      <c r="N61" s="14">
+        <f>IF(M61="","",G61*M61)</f>
+        <v/>
+      </c>
+      <c r="O61" s="11" t="inlineStr">
         <is>
           <t>From the same 100-piece set as the trigger pivot (20 of each length). Four per cover, from its outer face into M3 threads tapped 11 mm deep in the block and cap: 10 mm of thread, three times the 20 mm screw's. The kit's M3 x 20 would only reach 5</t>
         </is>
       </c>
-      <c r="P60" s="11" t="inlineStr">
+      <c r="P61" s="11" t="inlineStr">
         <is>
           <t>Base/README.md, Bought parts; user's M3 set 2026-10-24; Amazon listing 2026-10-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="21" t="n">
-        <v>43</v>
-      </c>
-      <c r="B61" s="22" t="inlineStr">
-        <is>
-          <t>Cable plug</t>
-        </is>
-      </c>
-      <c r="C61" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E61" s="21">
-        <f>ROUNDUP(C61*$C$3/D61,0)</f>
-        <v/>
-      </c>
-      <c r="F61" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G61" s="21">
-        <f>MAX(0,E61-F61)</f>
-        <v/>
-      </c>
-      <c r="H61" s="22" t="inlineStr">
-        <is>
-          <t>M2 x 12 countersunk screw</t>
-        </is>
-      </c>
-      <c r="I61" s="22" t="inlineStr">
-        <is>
-          <t>AvrestYPT</t>
-        </is>
-      </c>
-      <c r="J61" s="22" t="inlineStr"/>
-      <c r="K61" s="22" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="L61" s="24" t="inlineStr">
-        <is>
-          <t>B0FMD5TMSH</t>
-        </is>
-      </c>
-      <c r="M61" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N61" s="25">
-        <f>IF(M61="","",G61*M61)</f>
-        <v/>
-      </c>
-      <c r="O61" s="22" t="inlineStr">
-        <is>
-          <t>In the screw kit. Up from under the cable cover's rim, through a clearance hole, into an M2 thread tapped in the plug (1.6 mm pilot): pulls the plug that closes the cable's slot down onto the cover's shoulders. Length from the CAD</t>
-        </is>
-      </c>
-      <c r="P61" s="22" t="inlineStr">
-        <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
         </is>
       </c>
     </row>
@@ -3866,7 +3866,7 @@
       </c>
       <c r="B62" s="22" t="inlineStr">
         <is>
-          <t>Tube lock</t>
+          <t>Cable plug</t>
         </is>
       </c>
       <c r="C62" s="21" t="n">
@@ -3888,12 +3888,12 @@
       </c>
       <c r="H62" s="22" t="inlineStr">
         <is>
-          <t>M4 x 6 set screw</t>
+          <t>M2 x 12 countersunk screw</t>
         </is>
       </c>
       <c r="I62" s="22" t="inlineStr">
         <is>
-          <t>HIQTRADEBYJJ</t>
+          <t>AvrestYPT</t>
         </is>
       </c>
       <c r="J62" s="22" t="inlineStr"/>
@@ -3904,7 +3904,7 @@
       </c>
       <c r="L62" s="24" t="inlineStr">
         <is>
-          <t>B0DG33R714</t>
+          <t>B0FMD5TMSH</t>
         </is>
       </c>
       <c r="M62" s="25" t="n">
@@ -3916,77 +3916,67 @@
       </c>
       <c r="O62" s="22" t="inlineStr">
         <is>
-          <t>In the set screw kit. Tap the socket boss's 3.3 mm pilot M4; the tip goes into the tube's 4 mm lock hole, 38.5 mm from its bottom end</t>
+          <t>In the screw kit. Up from under the cable cover's rim, through a clearance hole, into an M2 thread tapped in the plug (1.6 mm pilot): pulls the plug that closes the cable's slot down onto the cover's shoulders. Length from the CAD</t>
         </is>
       </c>
       <c r="P62" s="22" t="inlineStr">
         <is>
-          <t>HIQTRADEBYJJ set screw kit (Amazon B0DG33R714); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="21" t="n">
+      <c r="A63" s="16" t="n">
         <v>45</v>
       </c>
-      <c r="B63" s="22" t="inlineStr">
+      <c r="B63" s="17" t="inlineStr">
         <is>
           <t>Friction knob</t>
         </is>
       </c>
-      <c r="C63" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D63" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E63" s="21">
+      <c r="C63" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="16">
         <f>ROUNDUP(C63*$C$3/D63,0)</f>
         <v/>
       </c>
-      <c r="F63" s="23" t="n">
+      <c r="F63" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="G63" s="21">
+      <c r="G63" s="16">
         <f>MAX(0,E63-F63)</f>
         <v/>
       </c>
-      <c r="H63" s="22" t="inlineStr">
-        <is>
-          <t>M5 x 20 countersunk screw + M5 hex nut</t>
-        </is>
-      </c>
-      <c r="I63" s="22" t="inlineStr">
-        <is>
-          <t>AvrestYPT</t>
-        </is>
-      </c>
-      <c r="J63" s="22" t="inlineStr"/>
-      <c r="K63" s="22" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="L63" s="24" t="inlineStr">
-        <is>
-          <t>B0FMD5TMSH</t>
-        </is>
-      </c>
-      <c r="M63" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N63" s="25">
+      <c r="H63" s="17" t="inlineStr">
+        <is>
+          <t>M5 x 16 hex-head bolt (ISO 4017 / DIN 933), zinc or stainless</t>
+        </is>
+      </c>
+      <c r="I63" s="17" t="inlineStr"/>
+      <c r="J63" s="17" t="inlineStr"/>
+      <c r="K63" s="17" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="L63" s="17" t="inlineStr"/>
+      <c r="M63" s="20" t="n"/>
+      <c r="N63" s="20">
         <f>IF(M63="","",G63*M63)</f>
         <v/>
       </c>
-      <c r="O63" s="22" t="inlineStr">
-        <is>
-          <t>In the screw kit. Glue the head into the printed knob (Base/stl/friction_knob.stl); the screw goes through the spring and the shoe into the nut, slid into the knob tower's slot from the front. Length from the CAD</t>
-        </is>
-      </c>
-      <c r="P63" s="22" t="inlineStr">
-        <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+      <c r="O63" s="17" t="inlineStr">
+        <is>
+          <t>CHECK: Not in the screw kits (they have only countersunk heads): any hardware store. Its head presses into the hex pocket moulded into the printed knob (Base/stl/friction_knob.stl), so the knob turns it; it goes through the spring and the shoe into the M5 nut</t>
+        </is>
+      </c>
+      <c r="P63" s="17" t="inlineStr">
+        <is>
+          <t>Base/README.md, Friction knob</t>
         </is>
       </c>
     </row>
@@ -3996,7 +3986,7 @@
       </c>
       <c r="B64" s="22" t="inlineStr">
         <is>
-          <t>Shoe hinge</t>
+          <t>Friction knob</t>
         </is>
       </c>
       <c r="C64" s="21" t="n">
@@ -4018,7 +4008,7 @@
       </c>
       <c r="H64" s="22" t="inlineStr">
         <is>
-          <t>M4 x 20 countersunk screw + M4 hex nut</t>
+          <t>M5 hex nut</t>
         </is>
       </c>
       <c r="I64" s="22" t="inlineStr">
@@ -4046,114 +4036,112 @@
       </c>
       <c r="O64" s="22" t="inlineStr">
         <is>
+          <t>In the screw kit. Slid into the knob tower's slot from the front; the friction bolt threads into it</t>
+        </is>
+      </c>
+      <c r="P64" s="22" t="inlineStr">
+        <is>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="21" t="n">
+        <v>47</v>
+      </c>
+      <c r="B65" s="22" t="inlineStr">
+        <is>
+          <t>Shoe hinge</t>
+        </is>
+      </c>
+      <c r="C65" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="21">
+        <f>ROUNDUP(C65*$C$3/D65,0)</f>
+        <v/>
+      </c>
+      <c r="F65" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="21">
+        <f>MAX(0,E65-F65)</f>
+        <v/>
+      </c>
+      <c r="H65" s="22" t="inlineStr">
+        <is>
+          <t>M4 x 20 countersunk screw + M4 hex nut</t>
+        </is>
+      </c>
+      <c r="I65" s="22" t="inlineStr">
+        <is>
+          <t>AvrestYPT</t>
+        </is>
+      </c>
+      <c r="J65" s="22" t="inlineStr"/>
+      <c r="K65" s="22" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L65" s="24" t="inlineStr">
+        <is>
+          <t>B0FMD5TMSH</t>
+        </is>
+      </c>
+      <c r="M65" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N65" s="25">
+        <f>IF(M65="","",G65*M65)</f>
+        <v/>
+      </c>
+      <c r="O65" s="22" t="inlineStr">
+        <is>
           <t>In the screw kit. Hinge pin through both frame lugs and the shoe's eye: head in the -y lug, nut in the +y lug's pocket (the lugs are 20 mm apart outside). Snug, then thread-lock: the shoe must still swing</t>
         </is>
       </c>
-      <c r="P64" s="22" t="inlineStr">
-        <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev4 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="M65" s="3" t="inlineStr">
+      <c r="P65" s="22" t="inlineStr">
+        <is>
+          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="M66" s="3" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="N65" s="15">
-        <f>SUM(N52:N64)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="7" t="inlineStr">
+      <c r="N66" s="15">
+        <f>SUM(N53:N65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
         <is>
           <t>Kits, consumables and tools</t>
         </is>
       </c>
-      <c r="B66" s="8" t="n"/>
-      <c r="C66" s="8" t="n"/>
-      <c r="D66" s="8" t="n"/>
-      <c r="E66" s="8" t="n"/>
-      <c r="F66" s="8" t="n"/>
-      <c r="G66" s="8" t="n"/>
-      <c r="H66" s="8" t="n"/>
-      <c r="I66" s="8" t="n"/>
-      <c r="J66" s="8" t="n"/>
-      <c r="K66" s="8" t="n"/>
-      <c r="L66" s="8" t="n"/>
-      <c r="M66" s="8" t="n"/>
-      <c r="N66" s="8" t="n"/>
-      <c r="O66" s="8" t="n"/>
-      <c r="P66" s="9" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="B67" s="11" t="inlineStr">
-        <is>
-          <t>Hardware</t>
-        </is>
-      </c>
-      <c r="C67" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D67" s="10" t="inlineStr">
-        <is>
-          <t>once</t>
-        </is>
-      </c>
-      <c r="E67" s="10">
-        <f>IF($C$3&gt;0,C67,0)</f>
-        <v/>
-      </c>
-      <c r="F67" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G67" s="10">
-        <f>MAX(0,E67-F67)</f>
-        <v/>
-      </c>
-      <c r="H67" s="11" t="inlineStr">
-        <is>
-          <t>Screw kit, 1715 pieces: countersunk hex-socket screws M2-M4 x 8, 12, 16, 20 and M5 x 10, 12, 16, 20, with hex nuts and washers, hex keys</t>
-        </is>
-      </c>
-      <c r="I67" s="11" t="inlineStr">
-        <is>
-          <t>AvrestYPT</t>
-        </is>
-      </c>
-      <c r="J67" s="11" t="inlineStr"/>
-      <c r="K67" s="11" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="L67" s="13" t="inlineStr">
-        <is>
-          <t>B0FMD5TMSH</t>
-        </is>
-      </c>
-      <c r="M67" s="14" t="n">
-        <v>17.99</v>
-      </c>
-      <c r="N67" s="14">
-        <f>IF(M67="","",G67*M67)</f>
-        <v/>
-      </c>
-      <c r="O67" s="11" t="inlineStr">
-        <is>
-          <t>Every countersunk screw and nut in the head and base (the green lines). Used: M3 x 12 (12), M3 x 20 (8), M4 x 12 (2), M4 x 16 (4), M4 x 20 (9), M5 x 20 (1); nuts M3 (4), M4 (17), M5 (1). Your order (link 2026-10-23)</t>
-        </is>
-      </c>
-      <c r="P67" s="11" t="inlineStr">
-        <is>
-          <t>Amazon listing 2026-10-23 (your order)</t>
-        </is>
-      </c>
+      <c r="B67" s="8" t="n"/>
+      <c r="C67" s="8" t="n"/>
+      <c r="D67" s="8" t="n"/>
+      <c r="E67" s="8" t="n"/>
+      <c r="F67" s="8" t="n"/>
+      <c r="G67" s="8" t="n"/>
+      <c r="H67" s="8" t="n"/>
+      <c r="I67" s="8" t="n"/>
+      <c r="J67" s="8" t="n"/>
+      <c r="K67" s="8" t="n"/>
+      <c r="L67" s="8" t="n"/>
+      <c r="M67" s="8" t="n"/>
+      <c r="N67" s="8" t="n"/>
+      <c r="O67" s="8" t="n"/>
+      <c r="P67" s="9" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="10" t="n">
@@ -4185,12 +4173,12 @@
       </c>
       <c r="H68" s="11" t="inlineStr">
         <is>
-          <t>Set screw kit, 500 pieces, 304 stainless: M3 x 3, 4, 5, 6; M4 x 4, 5, 6; M5 x 5, 8; M6 x 6, 10; M8 x 8; hex keys</t>
+          <t>Screw kit, 1715 pieces: countersunk hex-socket screws M2-M4 x 8, 12, 16, 20 and M5 x 10, 12, 16, 20, with hex nuts and washers, hex keys</t>
         </is>
       </c>
       <c r="I68" s="11" t="inlineStr">
         <is>
-          <t>HIQTRADEBYJJ</t>
+          <t>AvrestYPT</t>
         </is>
       </c>
       <c r="J68" s="11" t="inlineStr"/>
@@ -4201,11 +4189,11 @@
       </c>
       <c r="L68" s="13" t="inlineStr">
         <is>
-          <t>B0DG33R714</t>
+          <t>B0FMD5TMSH</t>
         </is>
       </c>
       <c r="M68" s="14" t="n">
-        <v>8.960000000000001</v>
+        <v>17.99</v>
       </c>
       <c r="N68" s="14">
         <f>IF(M68="","",G68*M68)</f>
@@ -4213,7 +4201,7 @@
       </c>
       <c r="O68" s="11" t="inlineStr">
         <is>
-          <t>The set screws: M5 x 8 (tube, head), M3 x 4 (trigger pull stop), M4 x 6 (tube lock, base). Your order (link 2026-10-23)</t>
+          <t>Every countersunk screw and nut in the head and base (the green lines). Used: M3 x 12 (4), M3 x 16 (8), M3 x 20 (8), M4 x 12 (2), M4 x 16 (4), M4 x 20 (9); nuts M3 (4), M4 (17), M5 (1). Your order (link 2026-10-23)</t>
         </is>
       </c>
       <c r="P68" s="11" t="inlineStr">
@@ -4228,7 +4216,7 @@
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C69" s="10" t="n">
@@ -4252,12 +4240,12 @@
       </c>
       <c r="H69" s="11" t="inlineStr">
         <is>
-          <t>White lithium grease, 1.5 oz tube</t>
+          <t>Set screw kit, 500 pieces, 304 stainless: M3 x 3, 4, 5, 6; M4 x 4, 5, 6; M5 x 5, 8; M6 x 6, 10; M8 x 8; hex keys</t>
         </is>
       </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
-          <t>Permatex</t>
+          <t>HIQTRADEBYJJ</t>
         </is>
       </c>
       <c r="J69" s="11" t="inlineStr"/>
@@ -4268,11 +4256,11 @@
       </c>
       <c r="L69" s="13" t="inlineStr">
         <is>
-          <t>B000HBNV58</t>
+          <t>B0DG33R714</t>
         </is>
       </c>
       <c r="M69" s="14" t="n">
-        <v>3.99</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="N69" s="14">
         <f>IF(M69="","",G69*M69)</f>
@@ -4280,12 +4268,12 @@
       </c>
       <c r="O69" s="11" t="inlineStr">
         <is>
-          <t>Bearing grease (not silicone paste)</t>
+          <t>The set screws: M5 x 8 (tube, head), M3 x 4 (trigger pull stop). Your order (link 2026-10-23)</t>
         </is>
       </c>
       <c r="P69" s="11" t="inlineStr">
         <is>
-          <t>Head/Rev4/README.md; Base/README.md; Amazon listing 2026-10-23</t>
+          <t>Amazon listing 2026-10-23 (your order)</t>
         </is>
       </c>
     </row>
@@ -4319,12 +4307,12 @@
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
-          <t>Silicone faucet grease, waterproof, 0.5 oz</t>
+          <t>White lithium grease, 1.5 oz tube</t>
         </is>
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>Danco</t>
+          <t>Permatex</t>
         </is>
       </c>
       <c r="J70" s="11" t="inlineStr"/>
@@ -4335,11 +4323,11 @@
       </c>
       <c r="L70" s="13" t="inlineStr">
         <is>
-          <t>B000DZFUPC</t>
+          <t>B000HBNV58</t>
         </is>
       </c>
       <c r="M70" s="14" t="n">
-        <v>5.68</v>
+        <v>3.99</v>
       </c>
       <c r="N70" s="14">
         <f>IF(M70="","",G70*M70)</f>
@@ -4347,12 +4335,12 @@
       </c>
       <c r="O70" s="11" t="inlineStr">
         <is>
-          <t>For the head's four throttle O-rings (grease them lightly before fitting)</t>
+          <t>Bearing grease (not silicone paste)</t>
         </is>
       </c>
       <c r="P70" s="11" t="inlineStr">
         <is>
-          <t>Head/Rev4/README.md; Amazon listing 2026-10-23</t>
+          <t>Head/Rev4/README.md; Base/README.md; Amazon listing 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -4386,31 +4374,27 @@
       </c>
       <c r="H71" s="11" t="inlineStr">
         <is>
-          <t>Solder paste, low-temperature (Sn42/Bi58, 138 C), syringe</t>
+          <t>Silicone faucet grease, waterproof, 0.5 oz</t>
         </is>
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>Chip Quik</t>
-        </is>
-      </c>
-      <c r="J71" s="11" t="inlineStr">
-        <is>
-          <t>NC191LT10</t>
-        </is>
-      </c>
+          <t>Danco</t>
+        </is>
+      </c>
+      <c r="J71" s="11" t="inlineStr"/>
       <c r="K71" s="11" t="inlineStr">
         <is>
-          <t>Digi-Key</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="L71" s="13" t="inlineStr">
         <is>
-          <t>315-NC191LT10-ND</t>
+          <t>B000DZFUPC</t>
         </is>
       </c>
       <c r="M71" s="14" t="n">
-        <v>7.95</v>
+        <v>5.68</v>
       </c>
       <c r="N71" s="14">
         <f>IF(M71="","",G71*M71)</f>
@@ -4418,12 +4402,12 @@
       </c>
       <c r="O71" s="11" t="inlineStr">
         <is>
-          <t>For the SMD parts on the board (U1, U2, the 1206 caps, the JST headers, SW1-SW3). Needs a hot plate or hot air tool and flux. Optional: hand-soldering works too</t>
+          <t>For the head's four throttle O-rings (grease them lightly before fitting)</t>
         </is>
       </c>
       <c r="P71" s="11" t="inlineStr">
         <is>
-          <t>Digi-Key cart 2026-10-23</t>
+          <t>Head/Rev4/README.md; Amazon listing 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -4457,17 +4441,17 @@
       </c>
       <c r="H72" s="11" t="inlineStr">
         <is>
-          <t>Tweezers, 1 mm tip (Olimex CHN-TWZ1MM), for placing the SMD parts</t>
+          <t>Solder paste, low-temperature (Sn42/Bi58, 138 C), syringe</t>
         </is>
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>Olimex</t>
+          <t>Chip Quik</t>
         </is>
       </c>
       <c r="J72" s="11" t="inlineStr">
         <is>
-          <t>CHN-TWZ1MM</t>
+          <t>NC191LT10</t>
         </is>
       </c>
       <c r="K72" s="11" t="inlineStr">
@@ -4477,11 +4461,11 @@
       </c>
       <c r="L72" s="13" t="inlineStr">
         <is>
-          <t>1188-CHN-TWZ1MM-ND</t>
+          <t>315-NC191LT10-ND</t>
         </is>
       </c>
       <c r="M72" s="14" t="n">
-        <v>0.82</v>
+        <v>7.95</v>
       </c>
       <c r="N72" s="14">
         <f>IF(M72="","",G72*M72)</f>
@@ -4489,61 +4473,132 @@
       </c>
       <c r="O72" s="11" t="inlineStr">
         <is>
+          <t>For the SMD parts on the board (U1, U2, the 1206 caps, the JST headers, SW1-SW3). Needs a hot plate or hot air tool and flux. Optional: hand-soldering works too</t>
+        </is>
+      </c>
+      <c r="P72" s="11" t="inlineStr">
+        <is>
+          <t>Digi-Key cart 2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B73" s="11" t="inlineStr">
+        <is>
+          <t>Assembly</t>
+        </is>
+      </c>
+      <c r="C73" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
+        <is>
+          <t>once</t>
+        </is>
+      </c>
+      <c r="E73" s="10">
+        <f>IF($C$3&gt;0,C73,0)</f>
+        <v/>
+      </c>
+      <c r="F73" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" s="10">
+        <f>MAX(0,E73-F73)</f>
+        <v/>
+      </c>
+      <c r="H73" s="11" t="inlineStr">
+        <is>
+          <t>Tweezers, 1 mm tip (Olimex CHN-TWZ1MM), for placing the SMD parts</t>
+        </is>
+      </c>
+      <c r="I73" s="11" t="inlineStr">
+        <is>
+          <t>Olimex</t>
+        </is>
+      </c>
+      <c r="J73" s="11" t="inlineStr">
+        <is>
+          <t>CHN-TWZ1MM</t>
+        </is>
+      </c>
+      <c r="K73" s="11" t="inlineStr">
+        <is>
+          <t>Digi-Key</t>
+        </is>
+      </c>
+      <c r="L73" s="13" t="inlineStr">
+        <is>
+          <t>1188-CHN-TWZ1MM-ND</t>
+        </is>
+      </c>
+      <c r="M73" s="14" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="N73" s="14">
+        <f>IF(M73="","",G73*M73)</f>
+        <v/>
+      </c>
+      <c r="O73" s="11" t="inlineStr">
+        <is>
           <t>Description from Olimex's sibling CHN-TWZ2MM listing: check the tip</t>
         </is>
       </c>
-      <c r="P72" s="11" t="inlineStr">
+      <c r="P73" s="11" t="inlineStr">
         <is>
           <t>Digi-Key order 102438510</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="M73" s="3" t="inlineStr">
+    <row r="74">
+      <c r="M74" s="3" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="N73" s="15">
-        <f>SUM(N67:N72)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="M75" s="3" t="inlineStr">
-        <is>
-          <t>Still to buy</t>
-        </is>
-      </c>
-      <c r="N75" s="15">
-        <f>N16+N20+N26+N29+N36+N50+N65+N73</f>
+      <c r="N74" s="15">
+        <f>SUM(N68:N73)</f>
         <v/>
       </c>
     </row>
     <row r="76">
       <c r="M76" s="3" t="inlineStr">
         <is>
-          <t>Whole build</t>
+          <t>Still to buy</t>
         </is>
       </c>
       <c r="N76" s="15">
-        <f>SUMPRODUCT(E6:E73,M6:M73)</f>
+        <f>N16+N20+N26+N29+N36+N51+N66+N74</f>
         <v/>
       </c>
     </row>
     <row r="77">
       <c r="M77" s="3" t="inlineStr">
         <is>
+          <t>Whole build</t>
+        </is>
+      </c>
+      <c r="N77" s="15">
+        <f>SUMPRODUCT(E6:E74,M6:M74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="M78" s="3" t="inlineStr">
+        <is>
           <t>Unpriced lines</t>
         </is>
       </c>
-      <c r="N77" s="3">
-        <f>COUNTIFS(A6:A73,"&gt;0",M6:M73,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="5" t="inlineStr">
+      <c r="N78" s="3">
+        <f>COUNTIFS(A6:A74,"&gt;0",M6:M74,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
         <is>
           <t>Still to buy counts the packs to order; whole build counts every pack needed, bought or not. Both leave out the unpriced lines: generic hardware and wire.</t>
         </is>
@@ -4551,16 +4606,16 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A51:P51"/>
-    <mergeCell ref="A66:P66"/>
     <mergeCell ref="A17:P17"/>
     <mergeCell ref="A37:P37"/>
     <mergeCell ref="A27:P27"/>
+    <mergeCell ref="A67:P67"/>
+    <mergeCell ref="A79:P79"/>
     <mergeCell ref="A6:P6"/>
     <mergeCell ref="D3:P3"/>
     <mergeCell ref="A30:P30"/>
-    <mergeCell ref="A78:P78"/>
     <mergeCell ref="A21:P21"/>
+    <mergeCell ref="A52:P52"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A2:P2"/>
   </mergeCells>
@@ -4598,7 +4653,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId37"/>
@@ -4609,14 +4664,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L60" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L61" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L62" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L63" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L64" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L68" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L64" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L68" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L73" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5470,7 +5525,7 @@
         </is>
       </c>
       <c r="C23" s="26">
-        <f>'Final BOM'!G47</f>
+        <f>'Final BOM'!G48</f>
         <v/>
       </c>
       <c r="D23" s="27" t="inlineStr">
@@ -5489,11 +5544,11 @@
         </is>
       </c>
       <c r="G23" s="30">
-        <f>'Final BOM'!M47</f>
+        <f>'Final BOM'!M48</f>
         <v/>
       </c>
       <c r="H23" s="30">
-        <f>IF('Final BOM'!M47="","",C23*G23)</f>
+        <f>IF('Final BOM'!M48="","",C23*G23)</f>
         <v/>
       </c>
       <c r="I23" s="27" t="inlineStr">
@@ -5512,7 +5567,7 @@
         </is>
       </c>
       <c r="C24" s="26">
-        <f>'Final BOM'!G71</f>
+        <f>'Final BOM'!G72</f>
         <v/>
       </c>
       <c r="D24" s="27" t="inlineStr">
@@ -5531,11 +5586,11 @@
         </is>
       </c>
       <c r="G24" s="30">
-        <f>'Final BOM'!M71</f>
+        <f>'Final BOM'!M72</f>
         <v/>
       </c>
       <c r="H24" s="30">
-        <f>IF('Final BOM'!M71="","",C24*G24)</f>
+        <f>IF('Final BOM'!M72="","",C24*G24)</f>
         <v/>
       </c>
       <c r="I24" s="27" t="inlineStr">
@@ -5554,7 +5609,7 @@
         </is>
       </c>
       <c r="C25" s="26">
-        <f>'Final BOM'!G72</f>
+        <f>'Final BOM'!G73</f>
         <v/>
       </c>
       <c r="D25" s="27" t="inlineStr">
@@ -5573,11 +5628,11 @@
         </is>
       </c>
       <c r="G25" s="30">
-        <f>'Final BOM'!M72</f>
+        <f>'Final BOM'!M73</f>
         <v/>
       </c>
       <c r="H25" s="30">
-        <f>IF('Final BOM'!M72="","",C25*G25)</f>
+        <f>IF('Final BOM'!M73="","",C25*G25)</f>
         <v/>
       </c>
       <c r="I25" s="27" t="inlineStr">
@@ -5705,7 +5760,7 @@
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-GripBearingCoupons.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-GripBearingCoupons.stl</t>
         </is>
       </c>
       <c r="D5" s="26" t="n">
@@ -5728,7 +5783,7 @@
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-ORingCoupon.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-ORingCoupon.stl</t>
         </is>
       </c>
       <c r="D6" s="26" t="n">
@@ -5751,7 +5806,7 @@
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-SensorSeatCoupon.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-SensorSeatCoupon.stl</t>
         </is>
       </c>
       <c r="D7" s="26" t="n">
@@ -5774,7 +5829,7 @@
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-Body.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-Body.stl</t>
         </is>
       </c>
       <c r="D8" s="26" t="n">
@@ -5797,7 +5852,7 @@
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-LowerPanel-Black.stl + -WhiteText.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-LowerPanel-Black.stl + -WhiteText.stl</t>
         </is>
       </c>
       <c r="D9" s="26" t="n">
@@ -5820,7 +5875,7 @@
       </c>
       <c r="C10" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-UpperPanel-Black.stl + -WhiteText.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-UpperPanel-Black.stl + -WhiteText.stl</t>
         </is>
       </c>
       <c r="D10" s="26" t="n">
@@ -5843,7 +5898,7 @@
       </c>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-Trigger.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-Trigger.stl</t>
         </is>
       </c>
       <c r="D11" s="26" t="n">
@@ -5866,7 +5921,7 @@
       </c>
       <c r="C12" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-Hat-Cap.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-Hat-Cap.stl</t>
         </is>
       </c>
       <c r="D12" s="26" t="n">
@@ -5889,7 +5944,7 @@
       </c>
       <c r="C13" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-Hat-RockerPlate.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-Hat-RockerPlate.stl</t>
         </is>
       </c>
       <c r="D13" s="26" t="n">
@@ -5912,7 +5967,7 @@
       </c>
       <c r="C14" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-Hat-Bezel.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-Hat-Bezel.stl</t>
         </is>
       </c>
       <c r="D14" s="26" t="n">
@@ -5935,7 +5990,7 @@
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-ThrottleGrip.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-ThrottleGrip.stl</t>
         </is>
       </c>
       <c r="D15" s="26" t="n">
@@ -5958,7 +6013,7 @@
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-FrictionCollar.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-FrictionCollar.stl</t>
         </is>
       </c>
       <c r="D16" s="26" t="n">
@@ -5981,7 +6036,7 @@
       </c>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-Pinion.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-Pinion.stl</t>
         </is>
       </c>
       <c r="D17" s="26" t="n">
@@ -6004,7 +6059,7 @@
       </c>
       <c r="C18" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4/stl/HueyHeadR4-MagnetShaft.stl</t>
+          <t>Head/Rev5/stl/HueyHeadR5-MagnetShaft.stl</t>
         </is>
       </c>
       <c r="D18" s="26" t="n">
@@ -6257,7 +6312,7 @@
       </c>
       <c r="E29" s="27" t="inlineStr">
         <is>
-          <t>Top face down; glue the M5 x 20's head into it</t>
+          <t>Top face down; the M5 x 16 hex bolt's head presses into its hex pocket</t>
         </is>
       </c>
     </row>
@@ -6383,7 +6438,7 @@
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
-          <t>Took an M6 hex head; the base now prints its own knob for the M5 x 20</t>
+          <t>Took an M6 hex head; the base now prints its own knob for an M5 x 16 hex bolt</t>
         </is>
       </c>
       <c r="E7" s="27" t="inlineStr">
@@ -6921,12 +6976,12 @@
       </c>
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>Head/Rev4</t>
+          <t>Head/Rev5</t>
         </is>
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>Current head design: Rev 4, one piece (Rev 3 with its neck block and trigger mount built back into the box). Rev 3 (Head/Rev3) is the same head in three parts, with no supports; Rev 2 (Head/) is superseded</t>
+          <t>Current head design: Rev 5, Rev 4 cut to the real UH-1 panels' dimensions, with printed threads. Rev 4 (Head/Rev4), the larger one-piece head it came from, is kept as a fallback</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Base Rev 3: M4 x 40 socket head cap lever screws, deeper friction nut
The lever halves take four M4 x 40 socket head cap screws (HELIFOUNER M4 x 30-50 kit) at x = +-17,
heads flush in counterbores at the top, nuts in hex pockets (corners along y) open to the
underside, so the seats are about 40 mm apart. Halves are chamfered after the split, skipping
the joint plane. The friction knob's M5 nut moves to the cap nuts' depth (z = -8.3) with an
M5 x 25 hex bolt. Renders, GLBs, README and BOM rebuilt.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/Heli_Collective_Final_BOM.xlsx
+++ b/BOM/Heli_Collective_Final_BOM.xlsx
@@ -3404,67 +3404,69 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="21" t="n">
+      <c r="A55" s="10" t="n">
         <v>37</v>
       </c>
-      <c r="B55" s="22" t="inlineStr">
+      <c r="B55" s="11" t="inlineStr">
         <is>
           <t>Lever halves</t>
         </is>
       </c>
-      <c r="C55" s="21" t="n">
+      <c r="C55" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="D55" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="21">
-        <f>ROUNDUP(C55*$C$3/D55,0)</f>
-        <v/>
-      </c>
-      <c r="F55" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="21">
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>once</t>
+        </is>
+      </c>
+      <c r="E55" s="10">
+        <f>IF($C$3&gt;0,C55,0)</f>
+        <v/>
+      </c>
+      <c r="F55" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="10">
         <f>MAX(0,E55-F55)</f>
         <v/>
       </c>
-      <c r="H55" s="22" t="inlineStr">
-        <is>
-          <t>M4 x 20 countersunk screw + M4 hex nut</t>
-        </is>
-      </c>
-      <c r="I55" s="22" t="inlineStr">
-        <is>
-          <t>AvrestYPT</t>
-        </is>
-      </c>
-      <c r="J55" s="22" t="inlineStr"/>
-      <c r="K55" s="22" t="inlineStr">
+      <c r="H55" s="11" t="inlineStr">
+        <is>
+          <t>Socket head cap screws M4 x 30 / 35 / 40 / 45 / 50, 12.9 black oxide, 10 of each, with 50 M4 nuts, flat and lock washers and a hex key (200 pieces)</t>
+        </is>
+      </c>
+      <c r="I55" s="11" t="inlineStr">
+        <is>
+          <t>HELIFOUNER</t>
+        </is>
+      </c>
+      <c r="J55" s="11" t="inlineStr"/>
+      <c r="K55" s="11" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="L55" s="24" t="inlineStr">
-        <is>
-          <t>B0FMD5TMSH</t>
-        </is>
-      </c>
-      <c r="M55" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N55" s="25">
+      <c r="L55" s="13" t="inlineStr">
+        <is>
+          <t>B0CDSKK7V1</t>
+        </is>
+      </c>
+      <c r="M55" s="14" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="N55" s="14">
         <f>IF(M55="","",G55*M55)</f>
         <v/>
       </c>
-      <c r="O55" s="22" t="inlineStr">
-        <is>
-          <t>In the screw kit. From the top, the heads 16 mm down their counterbores (a long 2.5 mm hex key helps); the nuts go in the lower half's pockets first</t>
-        </is>
-      </c>
-      <c r="P55" s="22" t="inlineStr">
-        <is>
-          <t>AvrestYPT screw kit (Amazon B0FMD5TMSH); Head/Rev5 and Base/mk3_rev3.py screw lists; renders/*Screws*.png</t>
+      <c r="O55" s="11" t="inlineStr">
+        <is>
+          <t>Uses 4 x M4 x 40, with 4 of its M4 nuts. The heads sit flush in 8 mm counterbores at the top and the nuts in hex pockets open to the underside, as far apart as the lever allows; no tip protrudes. The nuts go into the lower half's pockets first</t>
+        </is>
+      </c>
+      <c r="P55" s="11" t="inlineStr">
+        <is>
+          <t>Base/README.md, Bought parts; Amazon listing 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -3953,7 +3955,7 @@
       </c>
       <c r="H63" s="17" t="inlineStr">
         <is>
-          <t>M5 x 16 hex-head bolt (ISO 4017 / DIN 933), zinc or stainless</t>
+          <t>M5 x 25 hex-head bolt (ISO 4017 / DIN 933), zinc or stainless</t>
         </is>
       </c>
       <c r="I63" s="17" t="inlineStr"/>
@@ -4201,7 +4203,7 @@
       </c>
       <c r="O68" s="11" t="inlineStr">
         <is>
-          <t>Every countersunk screw and nut in the head and base (the green lines). Used: M3 x 12 (4), M3 x 16 (8), M3 x 20 (8), M4 x 12 (2), M4 x 16 (4), M4 x 20 (9); nuts M3 (4), M4 (17), M5 (1). Your order (link 2026-10-23)</t>
+          <t>Every countersunk screw and nut in the head and base (the green lines). Used: M3 x 12 (4), M3 x 16 (8), M3 x 20 (8), M4 x 12 (2), M4 x 16 (4), M4 x 20 (5); nuts M3 (4), M4 (13), M5 (1). Your order (link 2026-10-23)</t>
         </is>
       </c>
       <c r="P68" s="11" t="inlineStr">
@@ -6312,7 +6314,7 @@
       </c>
       <c r="E29" s="27" t="inlineStr">
         <is>
-          <t>Top face down; the M5 x 16 hex bolt's head presses into its hex pocket</t>
+          <t>Top face down; the M5 x 25 hex bolt's head presses into its hex pocket</t>
         </is>
       </c>
     </row>
@@ -6438,7 +6440,7 @@
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
-          <t>Took an M6 hex head; the base now prints its own knob for an M5 x 16 hex bolt</t>
+          <t>Took an M6 hex head; the base now prints its own knob for an M5 x 25 hex bolt</t>
         </is>
       </c>
       <c r="E7" s="27" t="inlineStr">

</xml_diff>

<commit_message>
Base Rev 3: two clamp screws on the strut collar
Two M4 x 12 + nuts, 20 mm apart, in place of one mid-ring. BOM, README and
renders updated (kit M4 x 12 2 -> 3, M4 nuts 13 -> 14).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/Heli_Collective_Final_BOM.xlsx
+++ b/BOM/Heli_Collective_Final_BOM.xlsx
@@ -3610,7 +3610,7 @@
         </is>
       </c>
       <c r="C58" s="21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D58" s="21" t="n">
         <v>1</v>
@@ -3656,7 +3656,7 @@
       </c>
       <c r="O58" s="22" t="inlineStr">
         <is>
-          <t>In the screw kit. Collar clamp: the head sits 2 mm into the -y ear, the nut in the +y ear's pocket</t>
+          <t>In the screw kit. Collar clamp, two 20 mm apart: each head sits 2 mm into the -y ear, its nut in the +y ear's pocket</t>
         </is>
       </c>
       <c r="P58" s="22" t="inlineStr">
@@ -4203,7 +4203,7 @@
       </c>
       <c r="O68" s="11" t="inlineStr">
         <is>
-          <t>Every countersunk screw and nut in the head and base (the green lines). Used: M3 x 12 (4), M3 x 16 (8), M3 x 20 (8), M4 x 12 (2), M4 x 16 (4), M4 x 20 (5); nuts M3 (4), M4 (13), M5 (1). Your order (link 2026-10-23)</t>
+          <t>Every countersunk screw and nut in the head and base (the green lines). Used: M3 x 12 (4), M3 x 16 (8), M3 x 20 (8), M4 x 12 (3), M4 x 16 (4), M4 x 20 (5); nuts M3 (4), M4 (14), M5 (1). Your order (link 2026-10-23)</t>
         </is>
       </c>
       <c r="P68" s="11" t="inlineStr">

</xml_diff>